<commit_message>
Update Exercise 2B and add Exercise 3B
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/netsanetaweke/Documents/DataAnalytics/week-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{936CCBC5-22EA-9648-9144-B4D2203CCA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CFF7D37-5C32-C641-B8AB-FE2CB2B885B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{AC28ED13-1875-C440-B8E0-8637456449D8}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="16520" windowHeight="21320" xr2:uid="{AC28ED13-1875-C440-B8E0-8637456449D8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>Name of data source</t>
   </si>
@@ -74,9 +74,6 @@
     <t>MBOX (emails);JSON (settings)</t>
   </si>
   <si>
-    <t>Google Takeout &gt; Deselect all &gt; Select Mail &gt; Next step &gt; Send download link via email &gt; Export once &gt; ZIP &gt; Create export &gt; Download from email when ready</t>
-  </si>
-  <si>
     <t>Reviewed export options; did not create an export or download data.</t>
   </si>
   <si>
@@ -108,6 +105,12 @@
   </si>
   <si>
     <t>Settings &amp; privacy &gt; Settings &gt; Accounts Center &gt; Your information and permissions &gt; Export your information &gt; Create export &gt; Select Facebook &gt; Export to device &gt; Choose options &gt; Start export &gt; Download when ready</t>
+  </si>
+  <si>
+    <t>E2</t>
+  </si>
+  <si>
+    <t>Open Google Takeout &gt; Deselect all &gt; Select Mail &gt; Next step &gt; Choose export options &gt; Create export &gt; Download when ready.</t>
   </si>
 </sst>
 </file>
@@ -494,12 +497,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBBAF406-43DD-1745-A3DA-4C31D4D6E695}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="75.6640625" customWidth="1"/>
+    <col min="3" max="3" width="104.33203125" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="129.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29.33203125" customWidth="1"/>
@@ -543,63 +546,68 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C5" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>